<commit_message>
Separate expense recipients from company paying accounts
</commit_message>
<xml_diff>
--- a/public/templates/BOH-expense.xlsx
+++ b/public/templates/BOH-expense.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entry" sheetId="1" r:id="Rd5181e59be5b407b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rd92c0f9dbed34389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entry" sheetId="1" r:id="Rb91848f33f6e46f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="Rd8987fc54d9548ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -42,12 +42,17 @@
       <x:name val="Arial"/>
     </x:font>
   </x:fonts>
-  <x:fills count="3">
+  <x:fills count="4">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0D3048"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -61,7 +66,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="11">
+  <x:cellXfs count="14">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -77,6 +82,11 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -85,8 +95,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EntryTable" displayName="EntryTable" ref="A1:I101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EntryTable" displayName="EntryTable" ref="A1:L101" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
     <x:tableColumn id="1" name="entryKey"/>
     <x:tableColumn id="2" name="payrollId"/>
     <x:tableColumn id="3" name="date"/>
@@ -94,8 +104,11 @@
     <x:tableColumn id="5" name="description"/>
     <x:tableColumn id="6" name="amount"/>
     <x:tableColumn id="7" name="account"/>
-    <x:tableColumn id="8" name="reference"/>
-    <x:tableColumn id="9" name="reconciled"/>
+    <x:tableColumn id="8" name="name"/>
+    <x:tableColumn id="9" name="recipientBank"/>
+    <x:tableColumn id="10" name="recipientAccount"/>
+    <x:tableColumn id="11" name="reference"/>
+    <x:tableColumn id="12" name="reconciled"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -308,6 +321,9 @@
     <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
@@ -332,10 +348,19 @@
       <x:c r="G1" s="4" t="str">
         <x:v>account</x:v>
       </x:c>
-      <x:c r="H1" s="4" t="str">
+      <x:c r="H1" s="11" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="I1" s="11" t="str">
+        <x:v>recipientBank</x:v>
+      </x:c>
+      <x:c r="J1" s="11" t="str">
+        <x:v>recipientAccount</x:v>
+      </x:c>
+      <x:c r="K1" s="11" t="str">
         <x:v>reference</x:v>
       </x:c>
-      <x:c r="I1" s="4" t="str">
+      <x:c r="L1" s="11" t="str">
         <x:v>reconciled</x:v>
       </x:c>
     </x:row>
@@ -349,6 +374,9 @@
       <x:c r="G2" s="5"/>
       <x:c r="H2" s="5"/>
       <x:c r="I2" s="5"/>
+      <x:c r="J2" s="5"/>
+      <x:c r="K2" s="5"/>
+      <x:c r="L2" s="5"/>
     </x:row>
     <x:row r="3" ht="24" customHeight="1">
       <x:c r="A3" s="5"/>
@@ -360,6 +388,9 @@
       <x:c r="G3" s="5"/>
       <x:c r="H3" s="5"/>
       <x:c r="I3" s="5"/>
+      <x:c r="J3" s="5"/>
+      <x:c r="K3" s="5"/>
+      <x:c r="L3" s="5"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="5"/>
@@ -371,6 +402,9 @@
       <x:c r="G4" s="5"/>
       <x:c r="H4" s="5"/>
       <x:c r="I4" s="5"/>
+      <x:c r="J4" s="5"/>
+      <x:c r="K4" s="5"/>
+      <x:c r="L4" s="5"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
       <x:c r="A5" s="5"/>
@@ -382,6 +416,9 @@
       <x:c r="G5" s="5"/>
       <x:c r="H5" s="5"/>
       <x:c r="I5" s="5"/>
+      <x:c r="J5" s="5"/>
+      <x:c r="K5" s="5"/>
+      <x:c r="L5" s="5"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
       <x:c r="A6" s="5"/>
@@ -393,6 +430,9 @@
       <x:c r="G6" s="5"/>
       <x:c r="H6" s="5"/>
       <x:c r="I6" s="5"/>
+      <x:c r="J6" s="5"/>
+      <x:c r="K6" s="5"/>
+      <x:c r="L6" s="5"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
       <x:c r="A7" s="5"/>
@@ -404,6 +444,9 @@
       <x:c r="G7" s="5"/>
       <x:c r="H7" s="5"/>
       <x:c r="I7" s="5"/>
+      <x:c r="J7" s="5"/>
+      <x:c r="K7" s="5"/>
+      <x:c r="L7" s="5"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
       <x:c r="A8" s="5"/>
@@ -415,6 +458,9 @@
       <x:c r="G8" s="5"/>
       <x:c r="H8" s="5"/>
       <x:c r="I8" s="5"/>
+      <x:c r="J8" s="5"/>
+      <x:c r="K8" s="5"/>
+      <x:c r="L8" s="5"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
       <x:c r="A9" s="5"/>
@@ -426,6 +472,9 @@
       <x:c r="G9" s="5"/>
       <x:c r="H9" s="5"/>
       <x:c r="I9" s="5"/>
+      <x:c r="J9" s="5"/>
+      <x:c r="K9" s="5"/>
+      <x:c r="L9" s="5"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
       <x:c r="A10" s="5"/>
@@ -437,6 +486,9 @@
       <x:c r="G10" s="5"/>
       <x:c r="H10" s="5"/>
       <x:c r="I10" s="5"/>
+      <x:c r="J10" s="5"/>
+      <x:c r="K10" s="5"/>
+      <x:c r="L10" s="5"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
       <x:c r="A11" s="5"/>
@@ -448,6 +500,9 @@
       <x:c r="G11" s="5"/>
       <x:c r="H11" s="5"/>
       <x:c r="I11" s="5"/>
+      <x:c r="J11" s="5"/>
+      <x:c r="K11" s="5"/>
+      <x:c r="L11" s="5"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
       <x:c r="A12" s="5"/>
@@ -459,6 +514,9 @@
       <x:c r="G12" s="5"/>
       <x:c r="H12" s="5"/>
       <x:c r="I12" s="5"/>
+      <x:c r="J12" s="5"/>
+      <x:c r="K12" s="5"/>
+      <x:c r="L12" s="5"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
       <x:c r="A13" s="5"/>
@@ -470,6 +528,9 @@
       <x:c r="G13" s="5"/>
       <x:c r="H13" s="5"/>
       <x:c r="I13" s="5"/>
+      <x:c r="J13" s="5"/>
+      <x:c r="K13" s="5"/>
+      <x:c r="L13" s="5"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="5"/>
@@ -481,6 +542,9 @@
       <x:c r="G14" s="5"/>
       <x:c r="H14" s="5"/>
       <x:c r="I14" s="5"/>
+      <x:c r="J14" s="5"/>
+      <x:c r="K14" s="5"/>
+      <x:c r="L14" s="5"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="5"/>
@@ -492,6 +556,9 @@
       <x:c r="G15" s="5"/>
       <x:c r="H15" s="5"/>
       <x:c r="I15" s="5"/>
+      <x:c r="J15" s="5"/>
+      <x:c r="K15" s="5"/>
+      <x:c r="L15" s="5"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="5"/>
@@ -503,6 +570,9 @@
       <x:c r="G16" s="5"/>
       <x:c r="H16" s="5"/>
       <x:c r="I16" s="5"/>
+      <x:c r="J16" s="5"/>
+      <x:c r="K16" s="5"/>
+      <x:c r="L16" s="5"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="5"/>
@@ -514,6 +584,9 @@
       <x:c r="G17" s="5"/>
       <x:c r="H17" s="5"/>
       <x:c r="I17" s="5"/>
+      <x:c r="J17" s="5"/>
+      <x:c r="K17" s="5"/>
+      <x:c r="L17" s="5"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="5"/>
@@ -525,6 +598,9 @@
       <x:c r="G18" s="5"/>
       <x:c r="H18" s="5"/>
       <x:c r="I18" s="5"/>
+      <x:c r="J18" s="5"/>
+      <x:c r="K18" s="5"/>
+      <x:c r="L18" s="5"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="5"/>
@@ -536,6 +612,9 @@
       <x:c r="G19" s="5"/>
       <x:c r="H19" s="5"/>
       <x:c r="I19" s="5"/>
+      <x:c r="J19" s="5"/>
+      <x:c r="K19" s="5"/>
+      <x:c r="L19" s="5"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="5"/>
@@ -547,6 +626,9 @@
       <x:c r="G20" s="5"/>
       <x:c r="H20" s="5"/>
       <x:c r="I20" s="5"/>
+      <x:c r="J20" s="5"/>
+      <x:c r="K20" s="5"/>
+      <x:c r="L20" s="5"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="5"/>
@@ -558,6 +640,9 @@
       <x:c r="G21" s="5"/>
       <x:c r="H21" s="5"/>
       <x:c r="I21" s="5"/>
+      <x:c r="J21" s="5"/>
+      <x:c r="K21" s="5"/>
+      <x:c r="L21" s="5"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="5"/>
@@ -569,6 +654,9 @@
       <x:c r="G22" s="5"/>
       <x:c r="H22" s="5"/>
       <x:c r="I22" s="5"/>
+      <x:c r="J22" s="5"/>
+      <x:c r="K22" s="5"/>
+      <x:c r="L22" s="5"/>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="5"/>
@@ -580,6 +668,9 @@
       <x:c r="G23" s="5"/>
       <x:c r="H23" s="5"/>
       <x:c r="I23" s="5"/>
+      <x:c r="J23" s="5"/>
+      <x:c r="K23" s="5"/>
+      <x:c r="L23" s="5"/>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="5"/>
@@ -591,6 +682,9 @@
       <x:c r="G24" s="5"/>
       <x:c r="H24" s="5"/>
       <x:c r="I24" s="5"/>
+      <x:c r="J24" s="5"/>
+      <x:c r="K24" s="5"/>
+      <x:c r="L24" s="5"/>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="5"/>
@@ -602,6 +696,9 @@
       <x:c r="G25" s="5"/>
       <x:c r="H25" s="5"/>
       <x:c r="I25" s="5"/>
+      <x:c r="J25" s="5"/>
+      <x:c r="K25" s="5"/>
+      <x:c r="L25" s="5"/>
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="5"/>
@@ -613,6 +710,9 @@
       <x:c r="G26" s="5"/>
       <x:c r="H26" s="5"/>
       <x:c r="I26" s="5"/>
+      <x:c r="J26" s="5"/>
+      <x:c r="K26" s="5"/>
+      <x:c r="L26" s="5"/>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
       <x:c r="A27" s="5"/>
@@ -624,6 +724,9 @@
       <x:c r="G27" s="5"/>
       <x:c r="H27" s="5"/>
       <x:c r="I27" s="5"/>
+      <x:c r="J27" s="5"/>
+      <x:c r="K27" s="5"/>
+      <x:c r="L27" s="5"/>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
       <x:c r="A28" s="5"/>
@@ -635,6 +738,9 @@
       <x:c r="G28" s="5"/>
       <x:c r="H28" s="5"/>
       <x:c r="I28" s="5"/>
+      <x:c r="J28" s="5"/>
+      <x:c r="K28" s="5"/>
+      <x:c r="L28" s="5"/>
     </x:row>
     <x:row r="29" ht="24" customHeight="1">
       <x:c r="A29" s="5"/>
@@ -646,6 +752,9 @@
       <x:c r="G29" s="5"/>
       <x:c r="H29" s="5"/>
       <x:c r="I29" s="5"/>
+      <x:c r="J29" s="5"/>
+      <x:c r="K29" s="5"/>
+      <x:c r="L29" s="5"/>
     </x:row>
     <x:row r="30" ht="24" customHeight="1">
       <x:c r="A30" s="5"/>
@@ -657,6 +766,9 @@
       <x:c r="G30" s="5"/>
       <x:c r="H30" s="5"/>
       <x:c r="I30" s="5"/>
+      <x:c r="J30" s="5"/>
+      <x:c r="K30" s="5"/>
+      <x:c r="L30" s="5"/>
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="5"/>
@@ -668,6 +780,9 @@
       <x:c r="G31" s="5"/>
       <x:c r="H31" s="5"/>
       <x:c r="I31" s="5"/>
+      <x:c r="J31" s="5"/>
+      <x:c r="K31" s="5"/>
+      <x:c r="L31" s="5"/>
     </x:row>
     <x:row r="32" ht="24" customHeight="1">
       <x:c r="A32" s="5"/>
@@ -679,6 +794,9 @@
       <x:c r="G32" s="5"/>
       <x:c r="H32" s="5"/>
       <x:c r="I32" s="5"/>
+      <x:c r="J32" s="5"/>
+      <x:c r="K32" s="5"/>
+      <x:c r="L32" s="5"/>
     </x:row>
     <x:row r="33" ht="24" customHeight="1">
       <x:c r="A33" s="5"/>
@@ -690,6 +808,9 @@
       <x:c r="G33" s="5"/>
       <x:c r="H33" s="5"/>
       <x:c r="I33" s="5"/>
+      <x:c r="J33" s="5"/>
+      <x:c r="K33" s="5"/>
+      <x:c r="L33" s="5"/>
     </x:row>
     <x:row r="34" ht="24" customHeight="1">
       <x:c r="A34" s="5"/>
@@ -701,6 +822,9 @@
       <x:c r="G34" s="5"/>
       <x:c r="H34" s="5"/>
       <x:c r="I34" s="5"/>
+      <x:c r="J34" s="5"/>
+      <x:c r="K34" s="5"/>
+      <x:c r="L34" s="5"/>
     </x:row>
     <x:row r="35" ht="24" customHeight="1">
       <x:c r="A35" s="5"/>
@@ -712,6 +836,9 @@
       <x:c r="G35" s="5"/>
       <x:c r="H35" s="5"/>
       <x:c r="I35" s="5"/>
+      <x:c r="J35" s="5"/>
+      <x:c r="K35" s="5"/>
+      <x:c r="L35" s="5"/>
     </x:row>
     <x:row r="36" ht="24" customHeight="1">
       <x:c r="A36" s="5"/>
@@ -723,6 +850,9 @@
       <x:c r="G36" s="5"/>
       <x:c r="H36" s="5"/>
       <x:c r="I36" s="5"/>
+      <x:c r="J36" s="5"/>
+      <x:c r="K36" s="5"/>
+      <x:c r="L36" s="5"/>
     </x:row>
     <x:row r="37" ht="24" customHeight="1">
       <x:c r="A37" s="5"/>
@@ -734,6 +864,9 @@
       <x:c r="G37" s="5"/>
       <x:c r="H37" s="5"/>
       <x:c r="I37" s="5"/>
+      <x:c r="J37" s="5"/>
+      <x:c r="K37" s="5"/>
+      <x:c r="L37" s="5"/>
     </x:row>
     <x:row r="38" ht="24" customHeight="1">
       <x:c r="A38" s="5"/>
@@ -745,6 +878,9 @@
       <x:c r="G38" s="5"/>
       <x:c r="H38" s="5"/>
       <x:c r="I38" s="5"/>
+      <x:c r="J38" s="5"/>
+      <x:c r="K38" s="5"/>
+      <x:c r="L38" s="5"/>
     </x:row>
     <x:row r="39" ht="24" customHeight="1">
       <x:c r="A39" s="5"/>
@@ -756,6 +892,9 @@
       <x:c r="G39" s="5"/>
       <x:c r="H39" s="5"/>
       <x:c r="I39" s="5"/>
+      <x:c r="J39" s="5"/>
+      <x:c r="K39" s="5"/>
+      <x:c r="L39" s="5"/>
     </x:row>
     <x:row r="40" ht="24" customHeight="1">
       <x:c r="A40" s="5"/>
@@ -767,6 +906,9 @@
       <x:c r="G40" s="5"/>
       <x:c r="H40" s="5"/>
       <x:c r="I40" s="5"/>
+      <x:c r="J40" s="5"/>
+      <x:c r="K40" s="5"/>
+      <x:c r="L40" s="5"/>
     </x:row>
     <x:row r="41" ht="24" customHeight="1">
       <x:c r="A41" s="5"/>
@@ -778,6 +920,9 @@
       <x:c r="G41" s="5"/>
       <x:c r="H41" s="5"/>
       <x:c r="I41" s="5"/>
+      <x:c r="J41" s="5"/>
+      <x:c r="K41" s="5"/>
+      <x:c r="L41" s="5"/>
     </x:row>
     <x:row r="42" ht="24" customHeight="1">
       <x:c r="A42" s="5"/>
@@ -789,6 +934,9 @@
       <x:c r="G42" s="5"/>
       <x:c r="H42" s="5"/>
       <x:c r="I42" s="5"/>
+      <x:c r="J42" s="5"/>
+      <x:c r="K42" s="5"/>
+      <x:c r="L42" s="5"/>
     </x:row>
     <x:row r="43" ht="24" customHeight="1">
       <x:c r="A43" s="5"/>
@@ -800,6 +948,9 @@
       <x:c r="G43" s="5"/>
       <x:c r="H43" s="5"/>
       <x:c r="I43" s="5"/>
+      <x:c r="J43" s="5"/>
+      <x:c r="K43" s="5"/>
+      <x:c r="L43" s="5"/>
     </x:row>
     <x:row r="44" ht="24" customHeight="1">
       <x:c r="A44" s="5"/>
@@ -811,6 +962,9 @@
       <x:c r="G44" s="5"/>
       <x:c r="H44" s="5"/>
       <x:c r="I44" s="5"/>
+      <x:c r="J44" s="5"/>
+      <x:c r="K44" s="5"/>
+      <x:c r="L44" s="5"/>
     </x:row>
     <x:row r="45" ht="24" customHeight="1">
       <x:c r="A45" s="5"/>
@@ -822,6 +976,9 @@
       <x:c r="G45" s="5"/>
       <x:c r="H45" s="5"/>
       <x:c r="I45" s="5"/>
+      <x:c r="J45" s="5"/>
+      <x:c r="K45" s="5"/>
+      <x:c r="L45" s="5"/>
     </x:row>
     <x:row r="46" ht="24" customHeight="1">
       <x:c r="A46" s="5"/>
@@ -833,6 +990,9 @@
       <x:c r="G46" s="5"/>
       <x:c r="H46" s="5"/>
       <x:c r="I46" s="5"/>
+      <x:c r="J46" s="5"/>
+      <x:c r="K46" s="5"/>
+      <x:c r="L46" s="5"/>
     </x:row>
     <x:row r="47" ht="24" customHeight="1">
       <x:c r="A47" s="5"/>
@@ -844,6 +1004,9 @@
       <x:c r="G47" s="5"/>
       <x:c r="H47" s="5"/>
       <x:c r="I47" s="5"/>
+      <x:c r="J47" s="5"/>
+      <x:c r="K47" s="5"/>
+      <x:c r="L47" s="5"/>
     </x:row>
     <x:row r="48" ht="24" customHeight="1">
       <x:c r="A48" s="5"/>
@@ -855,6 +1018,9 @@
       <x:c r="G48" s="5"/>
       <x:c r="H48" s="5"/>
       <x:c r="I48" s="5"/>
+      <x:c r="J48" s="5"/>
+      <x:c r="K48" s="5"/>
+      <x:c r="L48" s="5"/>
     </x:row>
     <x:row r="49" ht="24" customHeight="1">
       <x:c r="A49" s="5"/>
@@ -866,6 +1032,9 @@
       <x:c r="G49" s="5"/>
       <x:c r="H49" s="5"/>
       <x:c r="I49" s="5"/>
+      <x:c r="J49" s="5"/>
+      <x:c r="K49" s="5"/>
+      <x:c r="L49" s="5"/>
     </x:row>
     <x:row r="50" ht="24" customHeight="1">
       <x:c r="A50" s="5"/>
@@ -877,6 +1046,9 @@
       <x:c r="G50" s="5"/>
       <x:c r="H50" s="5"/>
       <x:c r="I50" s="5"/>
+      <x:c r="J50" s="5"/>
+      <x:c r="K50" s="5"/>
+      <x:c r="L50" s="5"/>
     </x:row>
     <x:row r="51" ht="24" customHeight="1">
       <x:c r="A51" s="5"/>
@@ -888,6 +1060,9 @@
       <x:c r="G51" s="5"/>
       <x:c r="H51" s="5"/>
       <x:c r="I51" s="5"/>
+      <x:c r="J51" s="5"/>
+      <x:c r="K51" s="5"/>
+      <x:c r="L51" s="5"/>
     </x:row>
     <x:row r="52" ht="24" customHeight="1">
       <x:c r="A52" s="5"/>
@@ -899,6 +1074,9 @@
       <x:c r="G52" s="5"/>
       <x:c r="H52" s="5"/>
       <x:c r="I52" s="5"/>
+      <x:c r="J52" s="5"/>
+      <x:c r="K52" s="5"/>
+      <x:c r="L52" s="5"/>
     </x:row>
     <x:row r="53" ht="24" customHeight="1">
       <x:c r="A53" s="5"/>
@@ -910,6 +1088,9 @@
       <x:c r="G53" s="5"/>
       <x:c r="H53" s="5"/>
       <x:c r="I53" s="5"/>
+      <x:c r="J53" s="5"/>
+      <x:c r="K53" s="5"/>
+      <x:c r="L53" s="5"/>
     </x:row>
     <x:row r="54" ht="24" customHeight="1">
       <x:c r="A54" s="5"/>
@@ -921,6 +1102,9 @@
       <x:c r="G54" s="5"/>
       <x:c r="H54" s="5"/>
       <x:c r="I54" s="5"/>
+      <x:c r="J54" s="5"/>
+      <x:c r="K54" s="5"/>
+      <x:c r="L54" s="5"/>
     </x:row>
     <x:row r="55" ht="24" customHeight="1">
       <x:c r="A55" s="5"/>
@@ -932,6 +1116,9 @@
       <x:c r="G55" s="5"/>
       <x:c r="H55" s="5"/>
       <x:c r="I55" s="5"/>
+      <x:c r="J55" s="5"/>
+      <x:c r="K55" s="5"/>
+      <x:c r="L55" s="5"/>
     </x:row>
     <x:row r="56" ht="24" customHeight="1">
       <x:c r="A56" s="5"/>
@@ -943,6 +1130,9 @@
       <x:c r="G56" s="5"/>
       <x:c r="H56" s="5"/>
       <x:c r="I56" s="5"/>
+      <x:c r="J56" s="5"/>
+      <x:c r="K56" s="5"/>
+      <x:c r="L56" s="5"/>
     </x:row>
     <x:row r="57" ht="24" customHeight="1">
       <x:c r="A57" s="5"/>
@@ -954,6 +1144,9 @@
       <x:c r="G57" s="5"/>
       <x:c r="H57" s="5"/>
       <x:c r="I57" s="5"/>
+      <x:c r="J57" s="5"/>
+      <x:c r="K57" s="5"/>
+      <x:c r="L57" s="5"/>
     </x:row>
     <x:row r="58" ht="24" customHeight="1">
       <x:c r="A58" s="5"/>
@@ -965,6 +1158,9 @@
       <x:c r="G58" s="5"/>
       <x:c r="H58" s="5"/>
       <x:c r="I58" s="5"/>
+      <x:c r="J58" s="5"/>
+      <x:c r="K58" s="5"/>
+      <x:c r="L58" s="5"/>
     </x:row>
     <x:row r="59" ht="24" customHeight="1">
       <x:c r="A59" s="5"/>
@@ -976,6 +1172,9 @@
       <x:c r="G59" s="5"/>
       <x:c r="H59" s="5"/>
       <x:c r="I59" s="5"/>
+      <x:c r="J59" s="5"/>
+      <x:c r="K59" s="5"/>
+      <x:c r="L59" s="5"/>
     </x:row>
     <x:row r="60" ht="24" customHeight="1">
       <x:c r="A60" s="5"/>
@@ -987,6 +1186,9 @@
       <x:c r="G60" s="5"/>
       <x:c r="H60" s="5"/>
       <x:c r="I60" s="5"/>
+      <x:c r="J60" s="5"/>
+      <x:c r="K60" s="5"/>
+      <x:c r="L60" s="5"/>
     </x:row>
     <x:row r="61" ht="24" customHeight="1">
       <x:c r="A61" s="5"/>
@@ -998,6 +1200,9 @@
       <x:c r="G61" s="5"/>
       <x:c r="H61" s="5"/>
       <x:c r="I61" s="5"/>
+      <x:c r="J61" s="5"/>
+      <x:c r="K61" s="5"/>
+      <x:c r="L61" s="5"/>
     </x:row>
     <x:row r="62" ht="24" customHeight="1">
       <x:c r="A62" s="5"/>
@@ -1009,6 +1214,9 @@
       <x:c r="G62" s="5"/>
       <x:c r="H62" s="5"/>
       <x:c r="I62" s="5"/>
+      <x:c r="J62" s="5"/>
+      <x:c r="K62" s="5"/>
+      <x:c r="L62" s="5"/>
     </x:row>
     <x:row r="63" ht="24" customHeight="1">
       <x:c r="A63" s="5"/>
@@ -1020,6 +1228,9 @@
       <x:c r="G63" s="5"/>
       <x:c r="H63" s="5"/>
       <x:c r="I63" s="5"/>
+      <x:c r="J63" s="5"/>
+      <x:c r="K63" s="5"/>
+      <x:c r="L63" s="5"/>
     </x:row>
     <x:row r="64" ht="24" customHeight="1">
       <x:c r="A64" s="5"/>
@@ -1031,6 +1242,9 @@
       <x:c r="G64" s="5"/>
       <x:c r="H64" s="5"/>
       <x:c r="I64" s="5"/>
+      <x:c r="J64" s="5"/>
+      <x:c r="K64" s="5"/>
+      <x:c r="L64" s="5"/>
     </x:row>
     <x:row r="65" ht="24" customHeight="1">
       <x:c r="A65" s="5"/>
@@ -1042,6 +1256,9 @@
       <x:c r="G65" s="5"/>
       <x:c r="H65" s="5"/>
       <x:c r="I65" s="5"/>
+      <x:c r="J65" s="5"/>
+      <x:c r="K65" s="5"/>
+      <x:c r="L65" s="5"/>
     </x:row>
     <x:row r="66" ht="24" customHeight="1">
       <x:c r="A66" s="5"/>
@@ -1053,6 +1270,9 @@
       <x:c r="G66" s="5"/>
       <x:c r="H66" s="5"/>
       <x:c r="I66" s="5"/>
+      <x:c r="J66" s="5"/>
+      <x:c r="K66" s="5"/>
+      <x:c r="L66" s="5"/>
     </x:row>
     <x:row r="67" ht="24" customHeight="1">
       <x:c r="A67" s="5"/>
@@ -1064,6 +1284,9 @@
       <x:c r="G67" s="5"/>
       <x:c r="H67" s="5"/>
       <x:c r="I67" s="5"/>
+      <x:c r="J67" s="5"/>
+      <x:c r="K67" s="5"/>
+      <x:c r="L67" s="5"/>
     </x:row>
     <x:row r="68" ht="24" customHeight="1">
       <x:c r="A68" s="5"/>
@@ -1075,6 +1298,9 @@
       <x:c r="G68" s="5"/>
       <x:c r="H68" s="5"/>
       <x:c r="I68" s="5"/>
+      <x:c r="J68" s="5"/>
+      <x:c r="K68" s="5"/>
+      <x:c r="L68" s="5"/>
     </x:row>
     <x:row r="69" ht="24" customHeight="1">
       <x:c r="A69" s="5"/>
@@ -1086,6 +1312,9 @@
       <x:c r="G69" s="5"/>
       <x:c r="H69" s="5"/>
       <x:c r="I69" s="5"/>
+      <x:c r="J69" s="5"/>
+      <x:c r="K69" s="5"/>
+      <x:c r="L69" s="5"/>
     </x:row>
     <x:row r="70" ht="24" customHeight="1">
       <x:c r="A70" s="5"/>
@@ -1097,6 +1326,9 @@
       <x:c r="G70" s="5"/>
       <x:c r="H70" s="5"/>
       <x:c r="I70" s="5"/>
+      <x:c r="J70" s="5"/>
+      <x:c r="K70" s="5"/>
+      <x:c r="L70" s="5"/>
     </x:row>
     <x:row r="71" ht="24" customHeight="1">
       <x:c r="A71" s="5"/>
@@ -1108,6 +1340,9 @@
       <x:c r="G71" s="5"/>
       <x:c r="H71" s="5"/>
       <x:c r="I71" s="5"/>
+      <x:c r="J71" s="5"/>
+      <x:c r="K71" s="5"/>
+      <x:c r="L71" s="5"/>
     </x:row>
     <x:row r="72" ht="24" customHeight="1">
       <x:c r="A72" s="5"/>
@@ -1119,6 +1354,9 @@
       <x:c r="G72" s="5"/>
       <x:c r="H72" s="5"/>
       <x:c r="I72" s="5"/>
+      <x:c r="J72" s="5"/>
+      <x:c r="K72" s="5"/>
+      <x:c r="L72" s="5"/>
     </x:row>
     <x:row r="73" ht="24" customHeight="1">
       <x:c r="A73" s="5"/>
@@ -1130,6 +1368,9 @@
       <x:c r="G73" s="5"/>
       <x:c r="H73" s="5"/>
       <x:c r="I73" s="5"/>
+      <x:c r="J73" s="5"/>
+      <x:c r="K73" s="5"/>
+      <x:c r="L73" s="5"/>
     </x:row>
     <x:row r="74" ht="24" customHeight="1">
       <x:c r="A74" s="5"/>
@@ -1141,6 +1382,9 @@
       <x:c r="G74" s="5"/>
       <x:c r="H74" s="5"/>
       <x:c r="I74" s="5"/>
+      <x:c r="J74" s="5"/>
+      <x:c r="K74" s="5"/>
+      <x:c r="L74" s="5"/>
     </x:row>
     <x:row r="75" ht="24" customHeight="1">
       <x:c r="A75" s="5"/>
@@ -1152,6 +1396,9 @@
       <x:c r="G75" s="5"/>
       <x:c r="H75" s="5"/>
       <x:c r="I75" s="5"/>
+      <x:c r="J75" s="5"/>
+      <x:c r="K75" s="5"/>
+      <x:c r="L75" s="5"/>
     </x:row>
     <x:row r="76" ht="24" customHeight="1">
       <x:c r="A76" s="5"/>
@@ -1163,6 +1410,9 @@
       <x:c r="G76" s="5"/>
       <x:c r="H76" s="5"/>
       <x:c r="I76" s="5"/>
+      <x:c r="J76" s="5"/>
+      <x:c r="K76" s="5"/>
+      <x:c r="L76" s="5"/>
     </x:row>
     <x:row r="77" ht="24" customHeight="1">
       <x:c r="A77" s="5"/>
@@ -1174,6 +1424,9 @@
       <x:c r="G77" s="5"/>
       <x:c r="H77" s="5"/>
       <x:c r="I77" s="5"/>
+      <x:c r="J77" s="5"/>
+      <x:c r="K77" s="5"/>
+      <x:c r="L77" s="5"/>
     </x:row>
     <x:row r="78" ht="24" customHeight="1">
       <x:c r="A78" s="5"/>
@@ -1185,6 +1438,9 @@
       <x:c r="G78" s="5"/>
       <x:c r="H78" s="5"/>
       <x:c r="I78" s="5"/>
+      <x:c r="J78" s="5"/>
+      <x:c r="K78" s="5"/>
+      <x:c r="L78" s="5"/>
     </x:row>
     <x:row r="79" ht="24" customHeight="1">
       <x:c r="A79" s="5"/>
@@ -1196,6 +1452,9 @@
       <x:c r="G79" s="5"/>
       <x:c r="H79" s="5"/>
       <x:c r="I79" s="5"/>
+      <x:c r="J79" s="5"/>
+      <x:c r="K79" s="5"/>
+      <x:c r="L79" s="5"/>
     </x:row>
     <x:row r="80" ht="24" customHeight="1">
       <x:c r="A80" s="5"/>
@@ -1207,6 +1466,9 @@
       <x:c r="G80" s="5"/>
       <x:c r="H80" s="5"/>
       <x:c r="I80" s="5"/>
+      <x:c r="J80" s="5"/>
+      <x:c r="K80" s="5"/>
+      <x:c r="L80" s="5"/>
     </x:row>
     <x:row r="81" ht="24" customHeight="1">
       <x:c r="A81" s="5"/>
@@ -1218,6 +1480,9 @@
       <x:c r="G81" s="5"/>
       <x:c r="H81" s="5"/>
       <x:c r="I81" s="5"/>
+      <x:c r="J81" s="5"/>
+      <x:c r="K81" s="5"/>
+      <x:c r="L81" s="5"/>
     </x:row>
     <x:row r="82" ht="24" customHeight="1">
       <x:c r="A82" s="5"/>
@@ -1229,6 +1494,9 @@
       <x:c r="G82" s="5"/>
       <x:c r="H82" s="5"/>
       <x:c r="I82" s="5"/>
+      <x:c r="J82" s="5"/>
+      <x:c r="K82" s="5"/>
+      <x:c r="L82" s="5"/>
     </x:row>
     <x:row r="83" ht="24" customHeight="1">
       <x:c r="A83" s="5"/>
@@ -1240,6 +1508,9 @@
       <x:c r="G83" s="5"/>
       <x:c r="H83" s="5"/>
       <x:c r="I83" s="5"/>
+      <x:c r="J83" s="5"/>
+      <x:c r="K83" s="5"/>
+      <x:c r="L83" s="5"/>
     </x:row>
     <x:row r="84" ht="24" customHeight="1">
       <x:c r="A84" s="5"/>
@@ -1251,6 +1522,9 @@
       <x:c r="G84" s="5"/>
       <x:c r="H84" s="5"/>
       <x:c r="I84" s="5"/>
+      <x:c r="J84" s="5"/>
+      <x:c r="K84" s="5"/>
+      <x:c r="L84" s="5"/>
     </x:row>
     <x:row r="85" ht="24" customHeight="1">
       <x:c r="A85" s="5"/>
@@ -1262,6 +1536,9 @@
       <x:c r="G85" s="5"/>
       <x:c r="H85" s="5"/>
       <x:c r="I85" s="5"/>
+      <x:c r="J85" s="5"/>
+      <x:c r="K85" s="5"/>
+      <x:c r="L85" s="5"/>
     </x:row>
     <x:row r="86" ht="24" customHeight="1">
       <x:c r="A86" s="5"/>
@@ -1273,6 +1550,9 @@
       <x:c r="G86" s="5"/>
       <x:c r="H86" s="5"/>
       <x:c r="I86" s="5"/>
+      <x:c r="J86" s="5"/>
+      <x:c r="K86" s="5"/>
+      <x:c r="L86" s="5"/>
     </x:row>
     <x:row r="87" ht="24" customHeight="1">
       <x:c r="A87" s="5"/>
@@ -1284,6 +1564,9 @@
       <x:c r="G87" s="5"/>
       <x:c r="H87" s="5"/>
       <x:c r="I87" s="5"/>
+      <x:c r="J87" s="5"/>
+      <x:c r="K87" s="5"/>
+      <x:c r="L87" s="5"/>
     </x:row>
     <x:row r="88" ht="24" customHeight="1">
       <x:c r="A88" s="5"/>
@@ -1295,6 +1578,9 @@
       <x:c r="G88" s="5"/>
       <x:c r="H88" s="5"/>
       <x:c r="I88" s="5"/>
+      <x:c r="J88" s="5"/>
+      <x:c r="K88" s="5"/>
+      <x:c r="L88" s="5"/>
     </x:row>
     <x:row r="89" ht="24" customHeight="1">
       <x:c r="A89" s="5"/>
@@ -1306,6 +1592,9 @@
       <x:c r="G89" s="5"/>
       <x:c r="H89" s="5"/>
       <x:c r="I89" s="5"/>
+      <x:c r="J89" s="5"/>
+      <x:c r="K89" s="5"/>
+      <x:c r="L89" s="5"/>
     </x:row>
     <x:row r="90" ht="24" customHeight="1">
       <x:c r="A90" s="5"/>
@@ -1317,6 +1606,9 @@
       <x:c r="G90" s="5"/>
       <x:c r="H90" s="5"/>
       <x:c r="I90" s="5"/>
+      <x:c r="J90" s="5"/>
+      <x:c r="K90" s="5"/>
+      <x:c r="L90" s="5"/>
     </x:row>
     <x:row r="91" ht="24" customHeight="1">
       <x:c r="A91" s="5"/>
@@ -1328,6 +1620,9 @@
       <x:c r="G91" s="5"/>
       <x:c r="H91" s="5"/>
       <x:c r="I91" s="5"/>
+      <x:c r="J91" s="5"/>
+      <x:c r="K91" s="5"/>
+      <x:c r="L91" s="5"/>
     </x:row>
     <x:row r="92" ht="24" customHeight="1">
       <x:c r="A92" s="5"/>
@@ -1339,6 +1634,9 @@
       <x:c r="G92" s="5"/>
       <x:c r="H92" s="5"/>
       <x:c r="I92" s="5"/>
+      <x:c r="J92" s="5"/>
+      <x:c r="K92" s="5"/>
+      <x:c r="L92" s="5"/>
     </x:row>
     <x:row r="93" ht="24" customHeight="1">
       <x:c r="A93" s="5"/>
@@ -1350,6 +1648,9 @@
       <x:c r="G93" s="5"/>
       <x:c r="H93" s="5"/>
       <x:c r="I93" s="5"/>
+      <x:c r="J93" s="5"/>
+      <x:c r="K93" s="5"/>
+      <x:c r="L93" s="5"/>
     </x:row>
     <x:row r="94" ht="24" customHeight="1">
       <x:c r="A94" s="5"/>
@@ -1361,6 +1662,9 @@
       <x:c r="G94" s="5"/>
       <x:c r="H94" s="5"/>
       <x:c r="I94" s="5"/>
+      <x:c r="J94" s="5"/>
+      <x:c r="K94" s="5"/>
+      <x:c r="L94" s="5"/>
     </x:row>
     <x:row r="95" ht="24" customHeight="1">
       <x:c r="A95" s="5"/>
@@ -1372,6 +1676,9 @@
       <x:c r="G95" s="5"/>
       <x:c r="H95" s="5"/>
       <x:c r="I95" s="5"/>
+      <x:c r="J95" s="5"/>
+      <x:c r="K95" s="5"/>
+      <x:c r="L95" s="5"/>
     </x:row>
     <x:row r="96" ht="24" customHeight="1">
       <x:c r="A96" s="5"/>
@@ -1383,6 +1690,9 @@
       <x:c r="G96" s="5"/>
       <x:c r="H96" s="5"/>
       <x:c r="I96" s="5"/>
+      <x:c r="J96" s="5"/>
+      <x:c r="K96" s="5"/>
+      <x:c r="L96" s="5"/>
     </x:row>
     <x:row r="97" ht="24" customHeight="1">
       <x:c r="A97" s="5"/>
@@ -1394,6 +1704,9 @@
       <x:c r="G97" s="5"/>
       <x:c r="H97" s="5"/>
       <x:c r="I97" s="5"/>
+      <x:c r="J97" s="5"/>
+      <x:c r="K97" s="5"/>
+      <x:c r="L97" s="5"/>
     </x:row>
     <x:row r="98" ht="24" customHeight="1">
       <x:c r="A98" s="5"/>
@@ -1405,6 +1718,9 @@
       <x:c r="G98" s="5"/>
       <x:c r="H98" s="5"/>
       <x:c r="I98" s="5"/>
+      <x:c r="J98" s="5"/>
+      <x:c r="K98" s="5"/>
+      <x:c r="L98" s="5"/>
     </x:row>
     <x:row r="99" ht="24" customHeight="1">
       <x:c r="A99" s="5"/>
@@ -1416,6 +1732,9 @@
       <x:c r="G99" s="5"/>
       <x:c r="H99" s="5"/>
       <x:c r="I99" s="5"/>
+      <x:c r="J99" s="5"/>
+      <x:c r="K99" s="5"/>
+      <x:c r="L99" s="5"/>
     </x:row>
     <x:row r="100" ht="24" customHeight="1">
       <x:c r="A100" s="5"/>
@@ -1427,6 +1746,9 @@
       <x:c r="G100" s="5"/>
       <x:c r="H100" s="5"/>
       <x:c r="I100" s="5"/>
+      <x:c r="J100" s="5"/>
+      <x:c r="K100" s="5"/>
+      <x:c r="L100" s="5"/>
     </x:row>
     <x:row r="101" ht="24" customHeight="1">
       <x:c r="A101" s="5"/>
@@ -1438,19 +1760,525 @@
       <x:c r="G101" s="5"/>
       <x:c r="H101" s="5"/>
       <x:c r="I101" s="5"/>
+      <x:c r="J101" s="5"/>
+      <x:c r="K101" s="5"/>
+      <x:c r="L101" s="5"/>
+    </x:row>
+    <x:row r="102">
+      <x:c r="H102" s="9"/>
+      <x:c r="I102" s="9"/>
+      <x:c r="J102" s="9"/>
+    </x:row>
+    <x:row r="103">
+      <x:c r="H103" s="9"/>
+      <x:c r="I103" s="9"/>
+      <x:c r="J103" s="9"/>
+    </x:row>
+    <x:row r="104">
+      <x:c r="H104" s="9"/>
+      <x:c r="I104" s="9"/>
+      <x:c r="J104" s="9"/>
+    </x:row>
+    <x:row r="105">
+      <x:c r="H105" s="9"/>
+      <x:c r="I105" s="9"/>
+      <x:c r="J105" s="9"/>
+    </x:row>
+    <x:row r="106">
+      <x:c r="H106" s="9"/>
+      <x:c r="I106" s="9"/>
+      <x:c r="J106" s="9"/>
+    </x:row>
+    <x:row r="107">
+      <x:c r="H107" s="9"/>
+      <x:c r="I107" s="9"/>
+      <x:c r="J107" s="9"/>
+    </x:row>
+    <x:row r="108">
+      <x:c r="H108" s="9"/>
+      <x:c r="I108" s="9"/>
+      <x:c r="J108" s="9"/>
+    </x:row>
+    <x:row r="109">
+      <x:c r="H109" s="9"/>
+      <x:c r="I109" s="9"/>
+      <x:c r="J109" s="9"/>
+    </x:row>
+    <x:row r="110">
+      <x:c r="H110" s="9"/>
+      <x:c r="I110" s="9"/>
+      <x:c r="J110" s="9"/>
+    </x:row>
+    <x:row r="111">
+      <x:c r="H111" s="9"/>
+      <x:c r="I111" s="9"/>
+      <x:c r="J111" s="9"/>
+    </x:row>
+    <x:row r="112">
+      <x:c r="H112" s="9"/>
+      <x:c r="I112" s="9"/>
+      <x:c r="J112" s="9"/>
+    </x:row>
+    <x:row r="113">
+      <x:c r="H113" s="9"/>
+      <x:c r="I113" s="9"/>
+      <x:c r="J113" s="9"/>
+    </x:row>
+    <x:row r="114">
+      <x:c r="H114" s="9"/>
+      <x:c r="I114" s="9"/>
+      <x:c r="J114" s="9"/>
+    </x:row>
+    <x:row r="115">
+      <x:c r="H115" s="9"/>
+      <x:c r="I115" s="9"/>
+      <x:c r="J115" s="9"/>
+    </x:row>
+    <x:row r="116">
+      <x:c r="H116" s="9"/>
+      <x:c r="I116" s="9"/>
+      <x:c r="J116" s="9"/>
+    </x:row>
+    <x:row r="117">
+      <x:c r="H117" s="9"/>
+      <x:c r="I117" s="9"/>
+      <x:c r="J117" s="9"/>
+    </x:row>
+    <x:row r="118">
+      <x:c r="H118" s="9"/>
+      <x:c r="I118" s="9"/>
+      <x:c r="J118" s="9"/>
+    </x:row>
+    <x:row r="119">
+      <x:c r="H119" s="9"/>
+      <x:c r="I119" s="9"/>
+      <x:c r="J119" s="9"/>
+    </x:row>
+    <x:row r="120">
+      <x:c r="H120" s="9"/>
+      <x:c r="I120" s="9"/>
+      <x:c r="J120" s="9"/>
+    </x:row>
+    <x:row r="121">
+      <x:c r="H121" s="9"/>
+      <x:c r="I121" s="9"/>
+      <x:c r="J121" s="9"/>
+    </x:row>
+    <x:row r="122">
+      <x:c r="H122" s="9"/>
+      <x:c r="I122" s="9"/>
+      <x:c r="J122" s="9"/>
+    </x:row>
+    <x:row r="123">
+      <x:c r="H123" s="9"/>
+      <x:c r="I123" s="9"/>
+      <x:c r="J123" s="9"/>
+    </x:row>
+    <x:row r="124">
+      <x:c r="H124" s="9"/>
+      <x:c r="I124" s="9"/>
+      <x:c r="J124" s="9"/>
+    </x:row>
+    <x:row r="125">
+      <x:c r="H125" s="9"/>
+      <x:c r="I125" s="9"/>
+      <x:c r="J125" s="9"/>
+    </x:row>
+    <x:row r="126">
+      <x:c r="H126" s="9"/>
+      <x:c r="I126" s="9"/>
+      <x:c r="J126" s="9"/>
+    </x:row>
+    <x:row r="127">
+      <x:c r="H127" s="9"/>
+      <x:c r="I127" s="9"/>
+      <x:c r="J127" s="9"/>
+    </x:row>
+    <x:row r="128">
+      <x:c r="H128" s="9"/>
+      <x:c r="I128" s="9"/>
+      <x:c r="J128" s="9"/>
+    </x:row>
+    <x:row r="129">
+      <x:c r="H129" s="9"/>
+      <x:c r="I129" s="9"/>
+      <x:c r="J129" s="9"/>
+    </x:row>
+    <x:row r="130">
+      <x:c r="H130" s="9"/>
+      <x:c r="I130" s="9"/>
+      <x:c r="J130" s="9"/>
+    </x:row>
+    <x:row r="131">
+      <x:c r="H131" s="9"/>
+      <x:c r="I131" s="9"/>
+      <x:c r="J131" s="9"/>
+    </x:row>
+    <x:row r="132">
+      <x:c r="H132" s="9"/>
+      <x:c r="I132" s="9"/>
+      <x:c r="J132" s="9"/>
+    </x:row>
+    <x:row r="133">
+      <x:c r="H133" s="9"/>
+      <x:c r="I133" s="9"/>
+      <x:c r="J133" s="9"/>
+    </x:row>
+    <x:row r="134">
+      <x:c r="H134" s="9"/>
+      <x:c r="I134" s="9"/>
+      <x:c r="J134" s="9"/>
+    </x:row>
+    <x:row r="135">
+      <x:c r="H135" s="9"/>
+      <x:c r="I135" s="9"/>
+      <x:c r="J135" s="9"/>
+    </x:row>
+    <x:row r="136">
+      <x:c r="H136" s="9"/>
+      <x:c r="I136" s="9"/>
+      <x:c r="J136" s="9"/>
+    </x:row>
+    <x:row r="137">
+      <x:c r="H137" s="9"/>
+      <x:c r="I137" s="9"/>
+      <x:c r="J137" s="9"/>
+    </x:row>
+    <x:row r="138">
+      <x:c r="H138" s="9"/>
+      <x:c r="I138" s="9"/>
+      <x:c r="J138" s="9"/>
+    </x:row>
+    <x:row r="139">
+      <x:c r="H139" s="9"/>
+      <x:c r="I139" s="9"/>
+      <x:c r="J139" s="9"/>
+    </x:row>
+    <x:row r="140">
+      <x:c r="H140" s="9"/>
+      <x:c r="I140" s="9"/>
+      <x:c r="J140" s="9"/>
+    </x:row>
+    <x:row r="141">
+      <x:c r="H141" s="9"/>
+      <x:c r="I141" s="9"/>
+      <x:c r="J141" s="9"/>
+    </x:row>
+    <x:row r="142">
+      <x:c r="H142" s="9"/>
+      <x:c r="I142" s="9"/>
+      <x:c r="J142" s="9"/>
+    </x:row>
+    <x:row r="143">
+      <x:c r="H143" s="9"/>
+      <x:c r="I143" s="9"/>
+      <x:c r="J143" s="9"/>
+    </x:row>
+    <x:row r="144">
+      <x:c r="H144" s="9"/>
+      <x:c r="I144" s="9"/>
+      <x:c r="J144" s="9"/>
+    </x:row>
+    <x:row r="145">
+      <x:c r="H145" s="9"/>
+      <x:c r="I145" s="9"/>
+      <x:c r="J145" s="9"/>
+    </x:row>
+    <x:row r="146">
+      <x:c r="H146" s="9"/>
+      <x:c r="I146" s="9"/>
+      <x:c r="J146" s="9"/>
+    </x:row>
+    <x:row r="147">
+      <x:c r="H147" s="9"/>
+      <x:c r="I147" s="9"/>
+      <x:c r="J147" s="9"/>
+    </x:row>
+    <x:row r="148">
+      <x:c r="H148" s="9"/>
+      <x:c r="I148" s="9"/>
+      <x:c r="J148" s="9"/>
+    </x:row>
+    <x:row r="149">
+      <x:c r="H149" s="9"/>
+      <x:c r="I149" s="9"/>
+      <x:c r="J149" s="9"/>
+    </x:row>
+    <x:row r="150">
+      <x:c r="H150" s="9"/>
+      <x:c r="I150" s="9"/>
+      <x:c r="J150" s="9"/>
+    </x:row>
+    <x:row r="151">
+      <x:c r="H151" s="9"/>
+      <x:c r="I151" s="9"/>
+      <x:c r="J151" s="9"/>
+    </x:row>
+    <x:row r="152">
+      <x:c r="H152" s="9"/>
+      <x:c r="I152" s="9"/>
+      <x:c r="J152" s="9"/>
+    </x:row>
+    <x:row r="153">
+      <x:c r="H153" s="9"/>
+      <x:c r="I153" s="9"/>
+      <x:c r="J153" s="9"/>
+    </x:row>
+    <x:row r="154">
+      <x:c r="H154" s="9"/>
+      <x:c r="I154" s="9"/>
+      <x:c r="J154" s="9"/>
+    </x:row>
+    <x:row r="155">
+      <x:c r="H155" s="9"/>
+      <x:c r="I155" s="9"/>
+      <x:c r="J155" s="9"/>
+    </x:row>
+    <x:row r="156">
+      <x:c r="H156" s="9"/>
+      <x:c r="I156" s="9"/>
+      <x:c r="J156" s="9"/>
+    </x:row>
+    <x:row r="157">
+      <x:c r="H157" s="9"/>
+      <x:c r="I157" s="9"/>
+      <x:c r="J157" s="9"/>
+    </x:row>
+    <x:row r="158">
+      <x:c r="H158" s="9"/>
+      <x:c r="I158" s="9"/>
+      <x:c r="J158" s="9"/>
+    </x:row>
+    <x:row r="159">
+      <x:c r="H159" s="9"/>
+      <x:c r="I159" s="9"/>
+      <x:c r="J159" s="9"/>
+    </x:row>
+    <x:row r="160">
+      <x:c r="H160" s="9"/>
+      <x:c r="I160" s="9"/>
+      <x:c r="J160" s="9"/>
+    </x:row>
+    <x:row r="161">
+      <x:c r="H161" s="9"/>
+      <x:c r="I161" s="9"/>
+      <x:c r="J161" s="9"/>
+    </x:row>
+    <x:row r="162">
+      <x:c r="H162" s="9"/>
+      <x:c r="I162" s="9"/>
+      <x:c r="J162" s="9"/>
+    </x:row>
+    <x:row r="163">
+      <x:c r="H163" s="9"/>
+      <x:c r="I163" s="9"/>
+      <x:c r="J163" s="9"/>
+    </x:row>
+    <x:row r="164">
+      <x:c r="H164" s="9"/>
+      <x:c r="I164" s="9"/>
+      <x:c r="J164" s="9"/>
+    </x:row>
+    <x:row r="165">
+      <x:c r="H165" s="9"/>
+      <x:c r="I165" s="9"/>
+      <x:c r="J165" s="9"/>
+    </x:row>
+    <x:row r="166">
+      <x:c r="H166" s="9"/>
+      <x:c r="I166" s="9"/>
+      <x:c r="J166" s="9"/>
+    </x:row>
+    <x:row r="167">
+      <x:c r="H167" s="9"/>
+      <x:c r="I167" s="9"/>
+      <x:c r="J167" s="9"/>
+    </x:row>
+    <x:row r="168">
+      <x:c r="H168" s="9"/>
+      <x:c r="I168" s="9"/>
+      <x:c r="J168" s="9"/>
+    </x:row>
+    <x:row r="169">
+      <x:c r="H169" s="9"/>
+      <x:c r="I169" s="9"/>
+      <x:c r="J169" s="9"/>
+    </x:row>
+    <x:row r="170">
+      <x:c r="H170" s="9"/>
+      <x:c r="I170" s="9"/>
+      <x:c r="J170" s="9"/>
+    </x:row>
+    <x:row r="171">
+      <x:c r="H171" s="9"/>
+      <x:c r="I171" s="9"/>
+      <x:c r="J171" s="9"/>
+    </x:row>
+    <x:row r="172">
+      <x:c r="H172" s="9"/>
+      <x:c r="I172" s="9"/>
+      <x:c r="J172" s="9"/>
+    </x:row>
+    <x:row r="173">
+      <x:c r="H173" s="9"/>
+      <x:c r="I173" s="9"/>
+      <x:c r="J173" s="9"/>
+    </x:row>
+    <x:row r="174">
+      <x:c r="H174" s="9"/>
+      <x:c r="I174" s="9"/>
+      <x:c r="J174" s="9"/>
+    </x:row>
+    <x:row r="175">
+      <x:c r="H175" s="9"/>
+      <x:c r="I175" s="9"/>
+      <x:c r="J175" s="9"/>
+    </x:row>
+    <x:row r="176">
+      <x:c r="H176" s="9"/>
+      <x:c r="I176" s="9"/>
+      <x:c r="J176" s="9"/>
+    </x:row>
+    <x:row r="177">
+      <x:c r="H177" s="9"/>
+      <x:c r="I177" s="9"/>
+      <x:c r="J177" s="9"/>
+    </x:row>
+    <x:row r="178">
+      <x:c r="H178" s="9"/>
+      <x:c r="I178" s="9"/>
+      <x:c r="J178" s="9"/>
+    </x:row>
+    <x:row r="179">
+      <x:c r="H179" s="9"/>
+      <x:c r="I179" s="9"/>
+      <x:c r="J179" s="9"/>
+    </x:row>
+    <x:row r="180">
+      <x:c r="H180" s="9"/>
+      <x:c r="I180" s="9"/>
+      <x:c r="J180" s="9"/>
+    </x:row>
+    <x:row r="181">
+      <x:c r="H181" s="9"/>
+      <x:c r="I181" s="9"/>
+      <x:c r="J181" s="9"/>
+    </x:row>
+    <x:row r="182">
+      <x:c r="H182" s="9"/>
+      <x:c r="I182" s="9"/>
+      <x:c r="J182" s="9"/>
+    </x:row>
+    <x:row r="183">
+      <x:c r="H183" s="9"/>
+      <x:c r="I183" s="9"/>
+      <x:c r="J183" s="9"/>
+    </x:row>
+    <x:row r="184">
+      <x:c r="H184" s="9"/>
+      <x:c r="I184" s="9"/>
+      <x:c r="J184" s="9"/>
+    </x:row>
+    <x:row r="185">
+      <x:c r="H185" s="9"/>
+      <x:c r="I185" s="9"/>
+      <x:c r="J185" s="9"/>
+    </x:row>
+    <x:row r="186">
+      <x:c r="H186" s="9"/>
+      <x:c r="I186" s="9"/>
+      <x:c r="J186" s="9"/>
+    </x:row>
+    <x:row r="187">
+      <x:c r="H187" s="9"/>
+      <x:c r="I187" s="9"/>
+      <x:c r="J187" s="9"/>
+    </x:row>
+    <x:row r="188">
+      <x:c r="H188" s="9"/>
+      <x:c r="I188" s="9"/>
+      <x:c r="J188" s="9"/>
+    </x:row>
+    <x:row r="189">
+      <x:c r="H189" s="9"/>
+      <x:c r="I189" s="9"/>
+      <x:c r="J189" s="9"/>
+    </x:row>
+    <x:row r="190">
+      <x:c r="H190" s="9"/>
+      <x:c r="I190" s="9"/>
+      <x:c r="J190" s="9"/>
+    </x:row>
+    <x:row r="191">
+      <x:c r="H191" s="9"/>
+      <x:c r="I191" s="9"/>
+      <x:c r="J191" s="9"/>
+    </x:row>
+    <x:row r="192">
+      <x:c r="H192" s="9"/>
+      <x:c r="I192" s="9"/>
+      <x:c r="J192" s="9"/>
+    </x:row>
+    <x:row r="193">
+      <x:c r="H193" s="9"/>
+      <x:c r="I193" s="9"/>
+      <x:c r="J193" s="9"/>
+    </x:row>
+    <x:row r="194">
+      <x:c r="H194" s="9"/>
+      <x:c r="I194" s="9"/>
+      <x:c r="J194" s="9"/>
+    </x:row>
+    <x:row r="195">
+      <x:c r="H195" s="9"/>
+      <x:c r="I195" s="9"/>
+      <x:c r="J195" s="9"/>
+    </x:row>
+    <x:row r="196">
+      <x:c r="H196" s="9"/>
+      <x:c r="I196" s="9"/>
+      <x:c r="J196" s="9"/>
+    </x:row>
+    <x:row r="197">
+      <x:c r="H197" s="9"/>
+      <x:c r="I197" s="9"/>
+      <x:c r="J197" s="9"/>
+    </x:row>
+    <x:row r="198">
+      <x:c r="H198" s="9"/>
+      <x:c r="I198" s="9"/>
+      <x:c r="J198" s="9"/>
+    </x:row>
+    <x:row r="199">
+      <x:c r="H199" s="9"/>
+      <x:c r="I199" s="9"/>
+      <x:c r="J199" s="9"/>
+    </x:row>
+    <x:row r="200">
+      <x:c r="H200" s="9"/>
+      <x:c r="I200" s="9"/>
+      <x:c r="J200" s="9"/>
+    </x:row>
+    <x:row r="201">
+      <x:c r="H201" s="9"/>
+      <x:c r="I201" s="9"/>
+      <x:c r="J201" s="9"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D2:D101">
       <x:formula1>"Payroll,Rent,Utilities,Teaching,Books,Marketing,Insurance,Bank fees,Office,Other"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="I2:I101">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="Paying account / Tài khoản chi" error="Choose Company BIDV or Company VCB. / Chọn Company BIDV hoặc Company VCB." sqref="G2:G201">
+      <x:formula1>"Company BIDV,Company VCB"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="L2:L101">
       <x:formula1>"true,false"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8d5e5ae202d14ae7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3467506e29c845a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1474,6 +2302,15 @@
         <x:v>BOH — Expenses paid / Chi phí đã thanh toán</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" ht="22" customHeight="1">
+      <x:c r="A3" s="1" t="str">
+        <x:v>Template version / Phiên bản: 2026-09-13</x:v>
+      </x:c>
+      <x:c r="B3" s="1"/>
+      <x:c r="C3" s="1"/>
+      <x:c r="D3" s="1"/>
+      <x:c r="E3" s="1"/>
+    </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="1" t="str">
         <x:v>Fill Entry from row 2. Keep headers unchanged. Maximum 200 rows. / Điền Entry từ dòng 2, giữ tên cột, tối đa 200 dòng.</x:v>
@@ -1485,7 +2322,7 @@
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="1" t="str">
-        <x:v>Examples below are guidance only; they are not imported. / Các ví dụ dưới đây không được nhập.</x:v>
+        <x:v>Examples below are fictional and are not imported. / Các ví dụ dưới đây là giả định và không được nhập.</x:v>
       </x:c>
       <x:c r="B5" s="1"/>
       <x:c r="C5" s="1"/>
@@ -1503,7 +2340,7 @@
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="1" t="str">
-        <x:v>Use exact names or IDs from the reference download. / Dùng tên chính xác hoặc mã trong danh sách tham chiếu.</x:v>
+        <x:v>Pay only from Company BIDV or Company VCB. / Chỉ chi từ Company BIDV hoặc Company VCB.</x:v>
       </x:c>
       <x:c r="B7" s="1"/>
       <x:c r="C7" s="1"/>
@@ -1529,7 +2366,9 @@
       <x:c r="E9" s="1"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
-      <x:c r="A10" s="1"/>
+      <x:c r="A10" s="1" t="str">
+        <x:v>Recipient details belong to the payee and may be blank. Name is required with bank details. / Có thể bỏ trống thông tin bên nhận tiền. Phải có tên người nhận khi nhập thông tin ngân hàng.</x:v>
+      </x:c>
       <x:c r="B10" s="1"/>
       <x:c r="C10" s="1"/>
       <x:c r="D10" s="1"/>
@@ -1657,13 +2496,13 @@
         <x:v>account</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Paying account / Tài khoản chi tiền</x:v>
+        <x:v>Company paying account / Tài khoản công ty chi tiền</x:v>
       </x:c>
       <x:c r="C18" s="10" t="str">
         <x:v>Yes / Có</x:v>
       </x:c>
       <x:c r="D18" s="10" t="str">
-        <x:v>Text / Văn bản</x:v>
+        <x:v>Company BIDV, Company VCB</x:v>
       </x:c>
       <x:c r="E18" s="5" t="str">
         <x:v>Company BIDV</x:v>
@@ -1671,33 +2510,84 @@
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
       <x:c r="A19" s="1" t="str">
-        <x:v>reference</x:v>
+        <x:v>name</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Invoice / reference</x:v>
+        <x:v>Recipient / account holder / Người nhận / Chủ tài khoản</x:v>
       </x:c>
       <x:c r="C19" s="10" t="str">
-        <x:v>No / Không</x:v>
+        <x:v>If bank details entered / Khi nhập thông tin ngân hàng</x:v>
       </x:c>
       <x:c r="D19" s="10" t="str">
         <x:v>Text / Văn bản</x:v>
       </x:c>
-      <x:c r="E19" s="5" t="str"/>
+      <x:c r="E19" s="5" t="str">
+        <x:v>Sample supplier</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
       <x:c r="A20" s="1" t="str">
-        <x:v>reconciled</x:v>
+        <x:v>recipientBank</x:v>
       </x:c>
       <x:c r="B20" s="10" t="str">
-        <x:v>Matched to bank statement / cash record</x:v>
+        <x:v>Recipient bank / Ngân hàng người nhận</x:v>
       </x:c>
       <x:c r="C20" s="10" t="str">
         <x:v>No / Không</x:v>
       </x:c>
       <x:c r="D20" s="10" t="str">
+        <x:v>Text / Văn bản</x:v>
+      </x:c>
+      <x:c r="E20" s="5" t="str">
+        <x:v>Example bank</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="1" t="str">
+        <x:v>recipientAccount</x:v>
+      </x:c>
+      <x:c r="B21" s="10" t="str">
+        <x:v>Recipient account number / Số tài khoản người nhận</x:v>
+      </x:c>
+      <x:c r="C21" s="10" t="str">
+        <x:v>No / Không</x:v>
+      </x:c>
+      <x:c r="D21" s="10" t="str">
+        <x:v>Text. Keep leading zeros. / Văn bản. Giữ số 0 ở đầu.</x:v>
+      </x:c>
+      <x:c r="E21" s="5" t="str">
+        <x:v>00123456789</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="48" customHeight="1">
+      <x:c r="A22" s="1" t="str">
+        <x:v>reference</x:v>
+      </x:c>
+      <x:c r="B22" s="10" t="str">
+        <x:v>Invoice / reference</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="str">
+        <x:v>No / Không</x:v>
+      </x:c>
+      <x:c r="D22" s="10" t="str">
+        <x:v>Text / Văn bản</x:v>
+      </x:c>
+      <x:c r="E22" s="5"/>
+    </x:row>
+    <x:row r="23" ht="48" customHeight="1">
+      <x:c r="A23" s="1" t="str">
+        <x:v>reconciled</x:v>
+      </x:c>
+      <x:c r="B23" s="10" t="str">
+        <x:v>Matched to bank statement / cash record</x:v>
+      </x:c>
+      <x:c r="C23" s="10" t="str">
+        <x:v>No / Không</x:v>
+      </x:c>
+      <x:c r="D23" s="10" t="str">
         <x:v>true / false</x:v>
       </x:c>
-      <x:c r="E20" s="5" t="str">
+      <x:c r="E23" s="5" t="str">
         <x:v>false</x:v>
       </x:c>
     </x:row>

</xml_diff>